<commit_message>
Correct the CBE rows in the print materials audit
The MBA and Marketing Analytics sheets print application windows
as month and day ranges with no year, so they do not go stale.
The reprint grounds are the printed version stamps instead:
VERSION: F25 on the MBA, Accountancy and Business Analytics
sheets, and Version: 24-25 on Marketing Analytics, which also
prints INTERIM PROGRAM COORDINATOR.

Business Analytics moves from no issues found to reprint.
Accountancy moves from verify to reprint, keeping the contact
address question. Fourteen reprint, six verify, one clean.

print-materials.md records the year-free window pattern and the
version stamps.
</commit_message>
<xml_diff>
--- a/committee/grad-facilitator/documents/print-materials-audit.xlsx
+++ b/committee/grad-facilitator/documents/print-materials-audit.xlsx
@@ -528,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -735,7 +735,19 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Two sheets break the rule and are marked reprint: MBA w Concentrations and Marketing Analytics.</t>
+          <t>Four CBE sheets print application windows. They are month and day ranges with no year attached, so they do not go stale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>version stamps</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Four CBE sheets print a version stamp on the page: F25 on the MBA, Accountancy and Business Analytics sheets, and 24-25 on Marketing Analytics. Those are printed dates and they do go stale.</t>
         </is>
       </c>
     </row>
@@ -844,7 +856,7 @@
       <c r="H2" s="8" t="inlineStr"/>
       <c r="I2" s="8" t="inlineStr">
         <is>
-          <t>dated F25 in the filename</t>
+          <t>dated F25 in the filename; no version stamp found on the page</t>
         </is>
       </c>
     </row>
@@ -920,13 +932,13 @@
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>prints an application deadlines block, against the rule that deadlines travel on the separate handout</t>
+          <t>prints VERSION: F25 on the page</t>
         </is>
       </c>
       <c r="H4" s="8" t="inlineStr"/>
       <c r="I4" s="8" t="inlineStr">
         <is>
-          <t>dated F25 in the filename</t>
+          <t>the application windows it prints (Fall October 1 to June 1, Spring August 1 to November 1, international a month earlier) carry no year and do not go stale; whether the sheet should carry them at all under the deadlines rule</t>
         </is>
       </c>
     </row>
@@ -954,20 +966,20 @@
       <c r="E5" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="F5" s="13" t="inlineStr">
-        <is>
-          <t>verify</t>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>reprint</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>prints jingwen-yang@csueastbay.edu with a hyphen</t>
+          <t>prints VERSION: F25 on the page</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr"/>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>the Graduate Program Info workbook gives jingwen.yang with a dot; one is wrong</t>
+          <t>prints jingwen-yang@csueastbay.edu with a hyphen; the Graduate Program Info workbook gives jingwen.yang with a dot, so one is wrong</t>
         </is>
       </c>
     </row>
@@ -995,18 +1007,18 @@
       <c r="E6" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>no issues found</t>
-        </is>
-      </c>
-      <c r="G6" s="8" t="inlineStr"/>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>reprint</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>prints Version: F25 on the page</t>
+        </is>
+      </c>
       <c r="H6" s="8" t="inlineStr"/>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>dated F25 in the filename</t>
-        </is>
-      </c>
+      <c r="I6" s="8" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -1039,13 +1051,13 @@
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>prints the international deadline offset, against the deadlines rule; dated January 2024</t>
+          <t>prints Version: 24-25, two cycles back; prints INTERIM PROGRAM COORDINATOR</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr"/>
       <c r="I7" s="8" t="inlineStr">
         <is>
-          <t>prints yi.he as contact; the workbook names Lan Wu as coordinator</t>
+          <t>prints yi.he as contact; the workbook names Lan Wu as coordinator. Its application windows carry no year and do not go stale</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add the page-read findings for three sheets
MS Statistics moves to a fuller reprint: its body names four
concentrations and omits Biostatistics, and it sends readers to a
Biostatistics chapter of the catalog as though Biostatistics were
a separate degree. It also prints a typo and a catalog phrase.

MS Special Education moves to reprint: the concentration name
appears two ways on one sheet.

Records that the course and unit comparison is not complete. The
sheets are set in two columns and extracted text interleaves
them, so 33 sheets still need reading page by page.

Fifteen reprint, six verify, four remove, twenty-four fix file.
</commit_message>
<xml_diff>
--- a/committee/grad-facilitator/documents/print-materials-audit.xlsx
+++ b/committee/grad-facilitator/documents/print-materials-audit.xlsx
@@ -528,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -704,48 +704,60 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n"/>
-      <c r="B18" s="2" t="n"/>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>course and unit drift</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Not completed. The sheets set their requirements in two columns and the extracted text interleaves them, so unit totals cannot be checked from the text. Three sheets were read page by page: Music, Statistics, and Special Education. The other 33 need the same treatment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>deadlines</t>
         </is>
       </c>
-      <c r="B19" s="5" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>rule</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Application deadlines stay off the per-program sheets. They travel on a separate dated handout, reprinted each cycle.</t>
-        </is>
-      </c>
+      <c r="B20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>exceptions</t>
+          <t>rule</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Four CBE sheets print application windows. They are month and day ranges with no year attached, so they do not go stale.</t>
+          <t>Application deadlines stay off the per-program sheets. They travel on a separate dated handout, reprinted each cycle.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
+          <t>exceptions</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Four CBE sheets print application windows. They are month and day ranges with no year attached, so they do not go stale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
           <t>version stamps</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Four CBE sheets print a version stamp on the page: F25 on the MBA, Accountancy and Business Analytics sheets, and 24-25 on Marketing Analytics. Those are printed dates and they do go stale.</t>
         </is>
@@ -1182,7 +1194,11 @@
           <t>catalog links point to catalog year 39; current catalog is 44</t>
         </is>
       </c>
-      <c r="I10" s="8" t="inlineStr"/>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>prints a comma before and in the program name; the catalog does not</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -1746,12 +1762,16 @@
       <c r="E25" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="F25" s="11" t="inlineStr">
-        <is>
-          <t>fix file</t>
-        </is>
-      </c>
-      <c r="G25" s="8" t="inlineStr"/>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>reprint</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>prints the concentration name two ways on one sheet, Mild/Moderate Support Needs and Mild-Moderate Support Needs; the catalog uses the first</t>
+        </is>
+      </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
           <t>catalog links point to catalog year 39; current catalog is 44</t>
@@ -2451,7 +2471,7 @@
       </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
-          <t>headed as one concentration while the filename and the QR index present it as the whole program; the catalog carries five concentrations</t>
+          <t>headed as one concentration while the filename and the QR index present it as the whole program; body names four concentrations and omits Biostatistics, where the catalog carries five; sends readers to the Biostatistics chapter of the catalog as though Biostatistics were a separate degree, which the catalog does not carry; prints the typo concentrations in in; prints the catalog phrase stated elsewhere in this catalog</t>
         </is>
       </c>
       <c r="H43" s="8" t="inlineStr">
@@ -2459,7 +2479,11 @@
           <t>catalog links point to catalog year 39; current catalog is 44</t>
         </is>
       </c>
-      <c r="I43" s="8" t="inlineStr"/>
+      <c r="I43" s="8" t="inlineStr">
+        <is>
+          <t>whether Biostatistics admits separately, which the Graduate Studies tile also implies</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Complete the unit total check across all 49 sheets
Columns are now separated by extracting glyph positions and
splitting each row at the page gutter, so requirements sections
and their course lines read in order.

Every declared section total was checked against the courses
beneath it. The Music capstone remains the only unit error.
Sheets with elective menus carry course units above their
declared totals by design and are not errors. Hospitality,
History and Statistics were read in full and are correct.

The History sheet prints "Repeat course three times for 12
units:" above its repeated course, which is the pattern the Music
sheet is missing.

Course titles and numbers remain unchecked against the catalog,
which blocks automated requests.
</commit_message>
<xml_diff>
--- a/committee/grad-facilitator/documents/print-materials-audit.xlsx
+++ b/committee/grad-facilitator/documents/print-materials-audit.xlsx
@@ -528,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -706,58 +706,70 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>course and unit drift</t>
+          <t>unit totals</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Not completed. The sheets set their requirements in two columns and the extracted text interleaves them, so unit totals cannot be checked from the text. Three sheets were read page by page: Music, Statistics, and Special Education. The other 33 need the same treatment.</t>
+          <t>Checked on all 49. Every declared section total was compared against the courses listed beneath it. The Music capstone is the only unit error. Sheets with elective menus carry course units above their declared total by design.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n"/>
-      <c r="B19" s="2" t="n"/>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>course titles</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Not checked against the catalog. The catalog blocks automated requests, so that comparison needs a person with a browser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="2" t="n"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>deadlines</t>
         </is>
       </c>
-      <c r="B20" s="5" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>rule</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Application deadlines stay off the per-program sheets. They travel on a separate dated handout, reprinted each cycle.</t>
-        </is>
-      </c>
+      <c r="B21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>exceptions</t>
+          <t>rule</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Four CBE sheets print application windows. They are month and day ranges with no year attached, so they do not go stale.</t>
+          <t>Application deadlines stay off the per-program sheets. They travel on a separate dated handout, reprinted each cycle.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
+          <t>exceptions</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Four CBE sheets print application windows. They are month and day ranges with no year attached, so they do not go stale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
           <t>version stamps</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Four CBE sheets print a version stamp on the page: F25 on the MBA, Accountancy and Business Analytics sheets, and 24-25 on Marketing Analytics. Those are printed dates and they do go stale.</t>
         </is>

</xml_diff>

<commit_message>
Drop the Music capstone from the print materials findings
MUS 693 is a 1-unit course taken three times. The sheet is
correct. MA Music returns to fix file, and the unit check across
all 49 sheets now records no unit errors.
</commit_message>
<xml_diff>
--- a/committee/grad-facilitator/documents/print-materials-audit.xlsx
+++ b/committee/grad-facilitator/documents/print-materials-audit.xlsx
@@ -711,7 +711,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Checked on all 49. Every declared section total was compared against the courses listed beneath it. The Music capstone is the only unit error. Sheets with elective menus carry course units above their declared total by design.</t>
+          <t>Checked on all 49. Every declared section total was compared against the courses listed beneath it. No unit errors. Sheets with elective menus carry course units above their declared total by design.</t>
         </is>
       </c>
     </row>
@@ -1273,16 +1273,12 @@
       <c r="E12" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="F12" s="12" t="inlineStr">
-        <is>
-          <t>reprint</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>capstone heading reads 3 units and the course line reads MUS 693 Capstone - Units: 1, with no note that it repeats three times</t>
-        </is>
-      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>fix file</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr"/>
       <c r="H12" s="8" t="inlineStr">
         <is>
           <t>catalog links point to catalog year 39; current catalog is 44; links to poid 18184, shared with seven other sheets</t>

</xml_diff>

<commit_message>
Name the embedded hyperlinks as such in the audit
Column H becomes "hyperlinks embedded in the PDF (digital only)".
The verdict "fix file" becomes "fix links", and the read me
defines it as a correct printed page whose embedded links point
somewhere wrong, reachable only when the file is shared
digitally.

print-materials.md retitles its catalog links section to match
and states where the links sit and when they reach a reader.
</commit_message>
<xml_diff>
--- a/committee/grad-facilitator/documents/print-materials-audit.xlsx
+++ b/committee/grad-facilitator/documents/print-materials-audit.xlsx
@@ -586,12 +586,12 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>The printed page is fine. Something in the file is wrong, which only shows when the PDF is opened rather than printed.</t>
+          <t>The printed page is correct and needs no reprint. Hyperlinks embedded in the PDF point somewhere wrong. A link shows nothing on paper, so this only reaches anyone when the file is shared digitally and clicked.</t>
         </is>
       </c>
     </row>
@@ -663,7 +663,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Read from the PDF link annotations. These are clickable in the file and invisible on the printed page.</t>
+          <t>Read from the link annotations embedded in each PDF. Most sit on the course lines. They are clickable when the file is opened and invisible on the printed page.</t>
         </is>
       </c>
     </row>
@@ -838,7 +838,7 @@
       </c>
       <c r="H1" s="7" t="inlineStr">
         <is>
-          <t>wrong in the file only</t>
+          <t>hyperlinks embedded in the PDF (digital only)</t>
         </is>
       </c>
       <c r="I1" s="7" t="inlineStr">
@@ -910,7 +910,7 @@
       </c>
       <c r="F3" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr"/>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr"/>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="F10" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr"/>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr"/>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr"/>
@@ -1312,7 +1312,7 @@
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr"/>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr"/>
@@ -1423,7 +1423,7 @@
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr"/>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr"/>
@@ -1497,7 +1497,7 @@
       </c>
       <c r="F18" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr"/>
@@ -1624,7 +1624,7 @@
       </c>
       <c r="F21" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr"/>
@@ -1661,7 +1661,7 @@
       </c>
       <c r="F22" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr"/>
@@ -1735,7 +1735,7 @@
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr"/>
@@ -1895,7 +1895,7 @@
       </c>
       <c r="F28" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr"/>
@@ -1973,7 +1973,7 @@
       </c>
       <c r="F30" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G30" s="8" t="inlineStr"/>
@@ -2010,7 +2010,7 @@
       </c>
       <c r="F31" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr"/>
@@ -2047,7 +2047,7 @@
       </c>
       <c r="F32" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G32" s="8" t="inlineStr"/>
@@ -2084,7 +2084,7 @@
       </c>
       <c r="F33" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr"/>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="F34" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G34" s="8" t="inlineStr"/>
@@ -2158,7 +2158,7 @@
       </c>
       <c r="F35" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G35" s="8" t="inlineStr"/>
@@ -2199,7 +2199,7 @@
       </c>
       <c r="F36" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G36" s="8" t="inlineStr"/>
@@ -2281,7 +2281,7 @@
       </c>
       <c r="F38" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G38" s="8" t="inlineStr"/>
@@ -2318,7 +2318,7 @@
       </c>
       <c r="F39" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G39" s="8" t="inlineStr"/>
@@ -2355,7 +2355,7 @@
       </c>
       <c r="F40" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G40" s="8" t="inlineStr"/>
@@ -2437,7 +2437,7 @@
       </c>
       <c r="F42" s="11" t="inlineStr">
         <is>
-          <t>fix file</t>
+          <t>fix links</t>
         </is>
       </c>
       <c r="G42" s="8" t="inlineStr"/>

</xml_diff>